<commit_message>
vault backup: 2026-04-27 01:16:50
</commit_message>
<xml_diff>
--- a/cartographie.xlsx
+++ b/cartographie.xlsx
@@ -2023,7 +2023,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -2065,7 +2065,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -2107,7 +2107,7 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Gi0/6</t>
+          <t>Gi1/2</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -2149,7 +2149,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Gi0/7</t>
+          <t>Gi1/3</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -2659,7 +2659,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -2701,7 +2701,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -2743,7 +2743,7 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Gi0/6</t>
+          <t>Gi1/2</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -2785,7 +2785,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Gi0/7</t>
+          <t>Gi1/3</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -3295,7 +3295,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -4183,7 +4183,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -4225,7 +4225,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -5071,7 +5071,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -5113,7 +5113,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -5959,7 +5959,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -6001,7 +6001,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>DIST-1 Gi0/4 ou Gi0/5</t>
+          <t>DIST-1 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>DIST-2 Gi0/4 ou Gi0/5</t>
+          <t>DIST-2 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>DIST-1 Gi0/4 ou Gi0/5</t>
+          <t>DIST-1 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>DIST-2 Gi0/4 ou Gi0/5</t>
+          <t>DIST-2 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>DIST-3 Gi0/4 ou Gi0/5</t>
+          <t>DIST-3 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>DIST-4 Gi0/4 ou Gi0/5</t>
+          <t>DIST-4 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Gi0/6</t>
+          <t>Gi1/2</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -8627,7 +8627,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Gi0/7</t>
+          <t>Gi1/3</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Gi0/6</t>
+          <t>Gi1/2</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Gi0/7</t>
+          <t>Gi1/3</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -9187,7 +9187,7 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -9427,7 +9427,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Gi0/4</t>
+          <t>Gi1/0</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Gi0/5</t>
+          <t>Gi1/1</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
@@ -11533,7 +11533,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>DIST-3 Gi0/4 ou Gi0/5</t>
+          <t>DIST-3 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>DIST-4 Gi0/4 ou Gi0/5</t>
+          <t>DIST-4 Gi1/0 ou Gi1/1</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-07-22 22:33:42
</commit_message>
<xml_diff>
--- a/cartographie.xlsx
+++ b/cartographie.xlsx
@@ -587,7 +587,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -627,7 +626,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>29 (8 LAN + 8 PROD + 5 DMZ + 6 ADMIN + 1 SOC + 1 MGMT)</t>
+          <t>38 identifiants : 31 de segmentation (8 LAN + 8 PROD + 5 DMZ + 7 ADMIN + 1 MGMT + 2 infra DC) + 3 système + 4 transit</t>
         </is>
       </c>
     </row>
@@ -639,7 +638,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>5 (PROD, DMZ, ADMIN, SOC, MGMT) + default underlay ; zone USERS = table globale LAN</t>
+          <t>4 VRF EVPN (PROD, DMZ, ADMIN, MGMT) + table globale underlay ; zone USERS = table globale du LAN Cisco</t>
         </is>
       </c>
     </row>
@@ -651,7 +650,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>~46 (loopbacks, liens /31, transit /30 ×5, VLAN /24, WAN+public, pfsync)</t>
+          <t>~48 (loopbacks, liens /31, transit /30 ×4, VLAN /24, MGMT ×3, WAN+public, pfsync)</t>
         </is>
       </c>
     </row>
@@ -735,35 +734,34 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>10.4.0.0/16</t>
+          <t>10.4.0.0/16 (VLAN 300-306, dont 306 ADMIN-SOC)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>DC SOC</t>
+          <t>MGMT</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>10.5.0.0/16 (VLAN 400, VRF-SOC)</t>
+          <t>10.254.0.0/24 (fabric DC) + 10.254.1.0/24 (LAN bloc 1) + 10.254.2.0/24 (LAN bloc 2)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>Blocs réservés</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>10.254.0.0/16 (VLAN 999 in-band)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+          <t>10.5.0.0/16 (promotion VRF-SOC) • 10.6.0.0/16 (VRF-PREPROD) — non déployés</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -839,7 +837,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>CORE-1/2 : interfaces routées, peer-link, loopback, SVI MGMT</t>
+          <t>CORE-1/2 : interfaces routées, peer-link, loopback (aucun SVI de management)</t>
         </is>
       </c>
     </row>
@@ -863,7 +861,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>ACC-1..4 : trunks Distribution + ports access + SVI MGMT</t>
+          <t>ACC-1..4 : trunks Distribution + ports access + SVI MGMT du bloc + ports parking</t>
         </is>
       </c>
     </row>
@@ -875,7 +873,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Bridges Linux, interface management, sous-bridges par zone</t>
+          <t>Bridges Linux, interface management, bridges par zone + cluster et migration</t>
         </is>
       </c>
     </row>
@@ -914,7 +912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -934,7 +932,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1050,8 +1047,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -1139,7 +1134,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF + source iBGP EVPN + VTEP</t>
+          <t>Router-ID OSPF + source iBGP EVPN + VTEP + administration in-band</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1245,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>300-305,400,999</t>
+          <t>300-306,990,991,999</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -1265,7 +1260,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Trunk vers HV (tous VLAN locaux)</t>
+          <t>Trunk vers HV (VLAN locaux + cluster/migration) — natif 997</t>
         </is>
       </c>
     </row>
@@ -1277,27 +1272,27 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>MGMT (VRF-MGMT)</t>
+          <t>MGMT (non raccordé)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>/24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>999</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1307,7 +1302,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Accès admin</t>
+          <t>Interface OOB non câblée dans la maquette : administration via Loopback0</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1428,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW ADMIN-MONITOR-PERF</t>
+          <t>Anycast GW ADMIN-OBSERV</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1561,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Vlan400</t>
+          <t>Vlan306</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -1576,7 +1571,7 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>10.5.0.1</t>
+          <t>10.4.36.1</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
@@ -1585,11 +1580,11 @@
         </is>
       </c>
       <c r="E28" s="10" t="n">
-        <v>400</v>
+        <v>306</v>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1599,7 +1594,47 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW SOC-CORE</t>
+          <t>Anycast GW ADMIN-SOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Vlan999</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>SVI anycast gateway</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>10.254.0.1</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>/24</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>999</v>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Anycast GW MGMT-DC — passerelle des hyperviseurs</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1757,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Vlan 999 (MGMT in-band uniquement)</t>
+          <t>Aucun — administration via Loopback0 (pas de SVI de management)</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1850,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band (SSH, syslog, SNMP sourcés dessus)</t>
         </is>
       </c>
     </row>
@@ -2198,46 +2233,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Vlan999</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>SVI MGMT</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>10.254.0.21</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>/24</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>MGMT</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Accès admin in-band</t>
-        </is>
-      </c>
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2358,7 +2361,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Vlan 999 (MGMT in-band uniquement)</t>
+          <t>Aucun — administration via Loopback0 (pas de SVI de management)</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2454,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band (SSH, syslog, SNMP sourcés dessus)</t>
         </is>
       </c>
     </row>
@@ -2834,46 +2837,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Vlan999</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>SVI MGMT</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>10.254.0.22</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>/24</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>MGMT</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Accès admin in-band</t>
-        </is>
-      </c>
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3087,7 +3058,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3295,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -3366,7 +3337,7 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -3413,7 +3384,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -3455,7 +3426,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3497,7 +3468,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -3539,7 +3510,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3581,7 +3552,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -3623,7 +3594,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3665,7 +3636,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -3707,7 +3678,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3729,12 +3700,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>SVI MGMT</t>
+          <t>SVI MGMT + VRRP</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.31</t>
+          <t>10.254.1.2</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -3742,10 +3713,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E31" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -3759,7 +3728,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Accès admin in-band</t>
+          <t>SVI management bloc 1 | VIP VRRP 10.254.1.1 | prio 120 | MASTER — passerelle des switches Access</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3944,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -4212,7 +4181,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -4254,7 +4223,7 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -4301,7 +4270,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -4343,7 +4312,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -4385,7 +4354,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -4427,7 +4396,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -4469,7 +4438,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -4511,7 +4480,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -4553,7 +4522,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -4595,7 +4564,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -4617,12 +4586,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>SVI MGMT</t>
+          <t>SVI MGMT + VRRP</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.32</t>
+          <t>10.254.1.3</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -4630,10 +4599,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E31" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -4647,7 +4614,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Accès admin in-band</t>
+          <t>SVI management bloc 1 | VIP VRRP 10.254.1.1 | prio 100 | BACKUP — passerelle des switches Access</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4830,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5067,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -5142,7 +5109,7 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -5189,7 +5156,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -5231,7 +5198,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -5273,7 +5240,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -5315,7 +5282,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -5357,7 +5324,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -5399,7 +5366,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -5441,7 +5408,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -5483,7 +5450,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -5505,12 +5472,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>SVI MGMT</t>
+          <t>SVI MGMT + VRRP</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.33</t>
+          <t>10.254.2.2</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -5518,10 +5485,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E31" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -5535,7 +5500,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Accès admin in-band</t>
+          <t>SVI management bloc 2 | VIP VRRP 10.254.2.1 | prio 120 | MASTER — passerelle des switches Access</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5716,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5953,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -6030,7 +5995,7 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -6077,7 +6042,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -6119,7 +6084,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -6161,7 +6126,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -6203,7 +6168,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -6245,7 +6210,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -6287,7 +6252,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -6329,7 +6294,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -6371,7 +6336,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>USERS</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -6393,12 +6358,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>SVI MGMT</t>
+          <t>SVI MGMT + VRRP</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.34</t>
+          <t>10.254.2.3</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -6406,10 +6371,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E31" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -6423,7 +6386,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Accès admin in-band</t>
+          <t>SVI management bloc 2 | VIP VRRP 10.254.2.1 | prio 100 | BACKUP — passerelle des switches Access</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6522,7 +6485,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Port-Security, DHCP Snooping, DAI, BPDU Guard, Storm Control</t>
+          <t>VTP transparent, VLAN natif dédié 997, ports inutilisés en VLAN 998 + shutdown, PortFast, BPDU Guard, Root Guard, Loop Guard, Port-Security, DHCP Snooping, DAI, IP Source Guard, Storm Control</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6587,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -6666,7 +6629,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -6740,7 +6703,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.41</t>
+          <t>10.254.1.41</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -6748,10 +6711,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E18" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -6765,7 +6726,47 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Accès admin équipement</t>
+          <t>Administration de l'équipement | ip default-gateway 10.254.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Ports non utilisés</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>L2 access (shutdown)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>998</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>VLAN PARKING : ports inutilisés affectés au VLAN 998 puis shutdown</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6864,7 +6865,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Port-Security, DHCP Snooping, DAI, BPDU Guard, Storm Control</t>
+          <t>VTP transparent, VLAN natif dédié 997, ports inutilisés en VLAN 998 + shutdown, PortFast, BPDU Guard, Root Guard, Loop Guard, Port-Security, DHCP Snooping, DAI, IP Source Guard, Storm Control</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6967,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -7008,7 +7009,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -7082,7 +7083,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.42</t>
+          <t>10.254.1.42</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -7090,10 +7091,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E18" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -7107,7 +7106,47 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Accès admin équipement</t>
+          <t>Administration de l'équipement | ip default-gateway 10.254.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Ports non utilisés</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>L2 access (shutdown)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>998</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>VLAN PARKING : ports inutilisés affectés au VLAN 998 puis shutdown</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7206,7 +7245,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Port-Security, DHCP Snooping, DAI, BPDU Guard, Storm Control</t>
+          <t>VTP transparent, VLAN natif dédié 997, ports inutilisés en VLAN 998 + shutdown, PortFast, BPDU Guard, Root Guard, Loop Guard, Port-Security, DHCP Snooping, DAI, IP Source Guard, Storm Control</t>
         </is>
       </c>
     </row>
@@ -7308,7 +7347,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -7350,7 +7389,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -7424,7 +7463,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.43</t>
+          <t>10.254.2.43</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -7432,10 +7471,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E18" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -7449,7 +7486,47 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Accès admin équipement</t>
+          <t>Administration de l'équipement | ip default-gateway 10.254.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Ports non utilisés</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>L2 access (shutdown)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>998</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>VLAN PARKING : ports inutilisés affectés au VLAN 998 puis shutdown</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7569,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -9231,7 +9307,7 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -9311,7 +9387,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -9391,7 +9467,7 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -9471,7 +9547,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -9711,7 +9787,7 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -9791,7 +9867,7 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
@@ -9871,7 +9947,7 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -9951,7 +10027,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>10,20,30,40,41,42,50,90,999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
@@ -10831,12 +10907,12 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>PROD/DMZ/ADMIN/SOC/MGMT</t>
+          <t>PROD/DMZ/ADMIN/MGMT</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
@@ -10851,7 +10927,7 @@
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>Trunk multi-VLAN multi-VRF, bridges vmbr-prod/dmz/admin/mgmt</t>
+          <t>Trunk multi-VLAN multi-VRF, bridges vmbr-prod/dmz/admin/cluster/migration/vmbr0</t>
         </is>
       </c>
     </row>
@@ -10911,12 +10987,12 @@
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>PROD/DMZ/ADMIN/SOC/MGMT</t>
+          <t>PROD/DMZ/ADMIN/MGMT</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr">
@@ -10991,12 +11067,12 @@
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>300-305,400,999</t>
+          <t>300-306,990,991,999</t>
         </is>
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>ADMIN/SOC/MGMT</t>
+          <t>ADMIN/MGMT</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
@@ -11011,7 +11087,7 @@
       </c>
       <c r="P46" s="5" t="inlineStr">
         <is>
-          <t>HV standalone management : PBS, PDM, QDevice, uniquement ADMIN+MGMT</t>
+          <t>HV standalone management : PBS, PDM, QDevice — ADMIN (dont SOC) + cluster + MGMT</t>
         </is>
       </c>
     </row>
@@ -11071,7 +11147,7 @@
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>4001-4005</t>
+          <t>4001-4004</t>
         </is>
       </c>
       <c r="M47" s="5" t="inlineStr">
@@ -11091,7 +11167,7 @@
       </c>
       <c r="P47" s="5" t="inlineStr">
         <is>
-          <t>Sous-interfaces em2.4001-4005 : transit PROD/DMZ/ADMIN/MGMT/SOC</t>
+          <t>Sous-interfaces em2.4001-4004 : transit PROD/DMZ/ADMIN/MGMT</t>
         </is>
       </c>
     </row>
@@ -11151,7 +11227,7 @@
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>4001-4005</t>
+          <t>4001-4004</t>
         </is>
       </c>
       <c r="M48" s="5" t="inlineStr">
@@ -11231,7 +11307,7 @@
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>4001-4005</t>
+          <t>4001-4004</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
@@ -11311,7 +11387,7 @@
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>4001-4005</t>
+          <t>4001-4004</t>
         </is>
       </c>
       <c r="M50" s="5" t="inlineStr">
@@ -11346,7 +11422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11430,7 +11506,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Port-Security, DHCP Snooping, DAI, BPDU Guard, Storm Control</t>
+          <t>VTP transparent, VLAN natif dédié 997, ports inutilisés en VLAN 998 + shutdown, PortFast, BPDU Guard, Root Guard, Loop Guard, Port-Security, DHCP Snooping, DAI, IP Source Guard, Storm Control</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11608,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -11574,7 +11650,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>all users + 999</t>
+          <t>10,20,30,40,41,42,50,90,999 (natif 997)</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -11648,7 +11724,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.44</t>
+          <t>10.254.2.44</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -11656,10 +11732,8 @@
           <t>/24</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="E18" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -11673,7 +11747,47 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Accès admin équipement</t>
+          <t>Administration de l'équipement | ip default-gateway 10.254.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Ports non utilisés</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>L2 access (shutdown)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>998</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>VLAN PARKING : ports inutilisés affectés au VLAN 998 puis shutdown</t>
         </is>
       </c>
     </row>
@@ -11688,7 +11802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11708,7 +11822,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -11796,7 +11909,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>PROD + DMZ + ADMIN + MGMT</t>
+          <t>PROD + DMZ + ADMIN (dont SOC) + cluster + MGMT</t>
         </is>
       </c>
     </row>
@@ -11812,8 +11925,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -11886,7 +11997,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -11901,7 +12012,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Trunk unique vers le Leaf</t>
+          <t>Trunk unique vers le Leaf — VLAN natif 997</t>
         </is>
       </c>
     </row>
@@ -11943,7 +12054,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006)</t>
+          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006) — GW anycast 10.254.0.1</t>
         </is>
       </c>
     </row>
@@ -12054,7 +12165,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>300-305</t>
+          <t>300-306</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -12069,19 +12180,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-ADMIN</t>
+          <t>Bridge pour VM VRF-ADMIN (dont VLAN 306 ADMIN-SOC)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>vmbr-soc</t>
+          <t>vmbr-cluster</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Bridge VLAN-aware SOC</t>
+          <t>Bridge VLAN-aware CLUSTER</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -12095,11 +12206,11 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>400</v>
+        <v>990</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>— (aucune VRF)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -12109,7 +12220,47 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-SOC (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
+          <t>Corosync du cluster Proxmox + QDevice — L2 pur, aucune SVI, non routable</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>vmbr-migration</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Bridge VLAN-aware MIGRATION</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>— (pas d'IP)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>991</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>— (aucune VRF)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Migration de VM et sauvegarde vers PBS — L2 pur, aucune SVI, non routable</t>
         </is>
       </c>
     </row>
@@ -12124,7 +12275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12144,7 +12295,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -12232,7 +12382,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>PROD + DMZ + ADMIN + MGMT</t>
+          <t>PROD + DMZ + ADMIN (dont SOC) + cluster + MGMT</t>
         </is>
       </c>
     </row>
@@ -12248,8 +12398,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -12322,7 +12470,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -12337,7 +12485,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Trunk unique vers le Leaf</t>
+          <t>Trunk unique vers le Leaf — VLAN natif 997</t>
         </is>
       </c>
     </row>
@@ -12379,7 +12527,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006)</t>
+          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006) — GW anycast 10.254.0.1</t>
         </is>
       </c>
     </row>
@@ -12490,7 +12638,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>300-305</t>
+          <t>300-306</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -12505,19 +12653,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-ADMIN</t>
+          <t>Bridge pour VM VRF-ADMIN (dont VLAN 306 ADMIN-SOC)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>vmbr-soc</t>
+          <t>vmbr-cluster</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Bridge VLAN-aware SOC</t>
+          <t>Bridge VLAN-aware CLUSTER</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -12531,11 +12679,11 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>400</v>
+        <v>990</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>— (aucune VRF)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -12545,7 +12693,47 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-SOC (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
+          <t>Corosync du cluster Proxmox + QDevice — L2 pur, aucune SVI, non routable</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>vmbr-migration</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Bridge VLAN-aware MIGRATION</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>— (pas d'IP)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>991</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>— (aucune VRF)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Migration de VM et sauvegarde vers PBS — L2 pur, aucune SVI, non routable</t>
         </is>
       </c>
     </row>
@@ -12560,7 +12748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12580,7 +12768,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -12668,7 +12855,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>ADMIN + MGMT uniquement</t>
+          <t>ADMIN (dont SOC) + cluster + MGMT uniquement</t>
         </is>
       </c>
     </row>
@@ -12684,8 +12871,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -12758,7 +12943,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>300-305,400,999</t>
+          <t>300-306,990,991,999</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -12773,7 +12958,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Trunk unique vers le Leaf</t>
+          <t>Trunk unique vers le Leaf — VLAN natif 997</t>
         </is>
       </c>
     </row>
@@ -12815,7 +13000,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006)</t>
+          <t>Interface admin de l'hyperviseur (SSH, webGUI 8006) — GW anycast 10.254.0.1</t>
         </is>
       </c>
     </row>
@@ -12842,7 +13027,7 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>300-305</t>
+          <t>300-306</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
@@ -12857,19 +13042,19 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-ADMIN (PBS, PDM)</t>
+          <t>Bridge pour VM VRF-ADMIN (dont VLAN 306 ADMIN-SOC)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>vmbr-soc</t>
+          <t>vmbr-cluster</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Bridge VLAN-aware SOC</t>
+          <t>Bridge VLAN-aware CLUSTER</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -12883,11 +13068,11 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>400</v>
+        <v>990</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>— (aucune VRF)</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -12897,7 +13082,47 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Bridge pour VM VRF-SOC (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
+          <t>Corosync du cluster Proxmox + QDevice — L2 pur, aucune SVI, non routable</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>vmbr-migration</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Bridge VLAN-aware MIGRATION</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>— (pas d'IP)</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>991</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>— (aucune VRF)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Migration de VM et sauvegarde vers PBS — L2 pur, aucune SVI, non routable</t>
         </is>
       </c>
     </row>
@@ -12932,7 +13157,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -12988,8 +13212,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -13448,7 +13670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13554,7 +13776,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Rouge clair (FFC7CE) — cellule SOC, VRF dédiée</t>
+          <t>Rouge clair (FFC7CE) — VLAN 306 ADMIN-SOC, au sein de VRF-ADMIN</t>
         </is>
       </c>
     </row>
@@ -13566,7 +13788,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Gris (D9D9D9) — VLAN 999 in-band</t>
+          <t>Gris (D9D9D9) — VLAN 999, trois domaines de diffusion distincts</t>
         </is>
       </c>
     </row>
@@ -13742,7 +13964,7 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>10.0.20.0/24 underlay + handoff VRF 10.0.21-25.x/30 (PROD/DMZ/ADMIN/MGMT/SOC), VLAN transit 4001-4005</t>
+          <t>10.0.20.0/24 underlay + handoff VRF 10.0.21-24.x/30 (PROD/DMZ/ADMIN/MGMT), VLAN transit 4001-4004</t>
         </is>
       </c>
     </row>
@@ -13850,7 +14072,7 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>10.254.0.0/24 unique</t>
+          <t>10.254.0.0/24 fabric DC (anycast Leaf) • 10.254.1.0/24 LAN bloc 1 • 10.254.2.0/24 LAN bloc 2 (VIP VRRP Dist)</t>
         </is>
       </c>
     </row>
@@ -13862,7 +14084,7 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>10.5.0.0/24 (VLAN 400) ; extensible 10.5.1+ pour granularité SIEM/NSM/TI/SIRP/SOAR</t>
+          <t>10.4.36.0/24 (VLAN 306, dans VRF-ADMIN) — 10.5.0.0/16 réservé si promotion en VRF</t>
         </is>
       </c>
     </row>
@@ -13895,6 +14117,42 @@
       <c r="B41" s="17" t="inlineStr">
         <is>
           <t>puis être répercutée ici, puis seulement ensuite configurée sur les équipements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>VLAN système</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>1 DEFAULT-UNUSED (élagué) • 997 NATIVE-UNUSED (natif des trunks) • 998 PARKING (ports inutilisés + shutdown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>VLAN infra DC</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
+          <t>990 DC-CLUSTER (corosync) • 991 DC-MIGRATION (migration VM + PBS) — L2 purs, sans SVI ni VRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Équipements L3 : Loopback0 routée. Switches Access (L2 pur) : SVI Vlan999 du bloc. Aucun réseau OOB.</t>
         </is>
       </c>
     </row>
@@ -13909,7 +14167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -13937,7 +14195,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -16718,7 +16975,7 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>ADMIN-MONITOR (Prometheus, Loki, Tempo, Grafana, Alloy)</t>
+          <t>ADMIN-OBSERV (Alloy, Prometheus, Loki, Tempo, Grafana)</t>
         </is>
       </c>
     </row>
@@ -16863,17 +17120,17 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>10.5.0.0/24</t>
+          <t>10.4.36.0/24</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>10.5.0.0</t>
+          <t>10.4.36.0</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>10.5.0.255</t>
+          <t>10.4.36.255</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
@@ -16883,20 +17140,20 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="G69" s="7" t="n">
-        <v>400</v>
+        <v>306</v>
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>10.5.0.1 AG</t>
+          <t>10.4.36.1 AG</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>SOC-CORE (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
+          <t>ADMIN-SOC (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
         </is>
       </c>
     </row>
@@ -16919,29 +17176,27 @@
           <t>10.254.0.255</t>
         </is>
       </c>
-      <c r="E70" s="15" t="inlineStr">
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>MGMT</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>MGMT</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
+      <c r="G70" s="7" t="n">
+        <v>999</v>
       </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
-          <t>10.254.0.254 VIP</t>
+          <t>10.254.0.1 AG</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Management in-band équipements</t>
+          <t>MGMT-DC — interfaces d'administration des hyperviseurs (VNI 10999)</t>
         </is>
       </c>
     </row>
@@ -16951,40 +17206,90 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>10.0.25.0/30</t>
+          <t>10.254.1.0/24</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>10.0.25.0</t>
+          <t>10.254.1.0</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>10.0.25.3</t>
-        </is>
-      </c>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>DC</t>
+          <t>10.254.1.255</t>
+        </is>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>LAN</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>MGMT-LAN</t>
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>4005</v>
+        <v>999</v>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>10.0.25.1 (VIP)</t>
+          <t>10.254.1.1 VIP VRRP</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Transit VRF-SOC FW ↔ Spine (VLAN 4005)</t>
+          <t>MGMT-LAN bloc 1 — SVI des ACC-1/ACC-2, passerelle sur DIST-1/DIST-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>10.254.2.0/24</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>10.254.2.0</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>10.254.2.255</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>LAN</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>MGMT-LAN</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>999</v>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>10.254.2.1 VIP VRRP</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>MGMT-LAN bloc 2 — SVI des ACC-3/ACC-4, passerelle sur DIST-3/DIST-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Note — VLAN sans sous-réseau : les VLAN 990 (DC-CLUSTER), 991 (DC-MIGRATION), 997 (NATIVE-UNUSED), 998 (PARKING) et 1 (DEFAULT-UNUSED) ne portent aucune interface L3 et n'apparaissent donc pas dans cette liste. Les blocs de transit 10.0.21-24.0/24 sont découpés en 4 /30 chacun ; seul le premier est listé ci-dessus, le détail complet figure dans l'onglet Liens-L3-Infra du plan d'adressage.</t>
         </is>
       </c>
     </row>
@@ -17019,7 +17324,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -17066,7 +17370,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Loopback OSPF</t>
+          <t>Loopback0 (OSPF + admin)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -17111,8 +17415,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -17788,7 +18090,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF, stable</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band (SSH + webGUI)</t>
         </is>
       </c>
     </row>
@@ -18045,84 +18347,24 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>em2.4005</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.2</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>SPINE-1 Et5.4005</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC vers Spine-1</t>
-        </is>
-      </c>
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>em3.4005</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.6</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>SPINE-2 Et5.4005</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC vers Spine-2</t>
-        </is>
-      </c>
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18155,7 +18397,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -18202,7 +18443,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Loopback OSPF</t>
+          <t>Loopback0 (OSPF + admin)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -18235,8 +18476,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -18912,7 +19151,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF</t>
+          <t>Router-ID OSPF ET adresse d'administration in-band (SSH + webGUI)</t>
         </is>
       </c>
     </row>
@@ -19211,84 +19450,24 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>em2.4005</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.10</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>SPINE-1 Et6.4005</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC vers Spine-1</t>
-        </is>
-      </c>
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>em3.4005</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.14</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>SPINE-2 Et6.4005</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC vers Spine-2</t>
-        </is>
-      </c>
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19321,7 +19500,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -19425,8 +19603,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -19514,7 +19690,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF + source iBGP EVPN</t>
+          <t>Router-ID OSPF + source iBGP EVPN + adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -19652,7 +19828,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>L3 /31 + trunk 4001-4005</t>
+          <t>L3 /31 + trunk 4001-4004</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -19862,7 +20038,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>L3 /31 + trunk 4001-4005</t>
+          <t>L3 /31 + trunk 4001-4004</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -20072,27 +20248,27 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>MGMT (VRF-MGMT)</t>
+          <t>MGMT (non raccordé)</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>/24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>999</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -20102,89 +20278,29 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Accès admin</t>
+          <t>Interface OOB non câblée dans la maquette : administration via Loopback0</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Ethernet5.4005</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.1</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>FW-1 em2.4005</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC (VIP Anycast) vers FW-1</t>
-        </is>
-      </c>
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Ethernet6.4005</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.9</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>FW-2 em2.4005</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC (VIP Anycast) vers FW-2</t>
-        </is>
-      </c>
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20217,7 +20333,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -20321,8 +20436,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -20410,7 +20523,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF + source iBGP EVPN</t>
+          <t>Router-ID OSPF + source iBGP EVPN + adresse d'administration in-band</t>
         </is>
       </c>
     </row>
@@ -20548,7 +20661,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>L3 /31 + trunk 4001-4005</t>
+          <t>L3 /31 + trunk 4001-4004</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -20758,7 +20871,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>L3 /31 + trunk 4001-4005</t>
+          <t>L3 /31 + trunk 4001-4004</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -20968,27 +21081,27 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>MGMT (VRF-MGMT)</t>
+          <t>MGMT (non raccordé)</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>/24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>999</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -20998,89 +21111,29 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Accès admin</t>
+          <t>Interface OOB non câblée dans la maquette : administration via Loopback0</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Ethernet5.4005</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.5</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>FW-1 em3.4005</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC (VIP Anycast) vers FW-1</t>
-        </is>
-      </c>
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Ethernet6.4005</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Sub-if trunk 802.1Q</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>10.0.25.13</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>/30</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="n">
-        <v>4005</v>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>SOC</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>FW-2 em3.4005</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Transit VRF-SOC (VIP Anycast) vers FW-2</t>
-        </is>
-      </c>
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21093,7 +21146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21113,7 +21166,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -21229,8 +21281,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -21318,7 +21368,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF + source iBGP EVPN + VTEP</t>
+          <t>Router-ID OSPF + source iBGP EVPN + VTEP + administration in-band</t>
         </is>
       </c>
     </row>
@@ -21429,7 +21479,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -21444,7 +21494,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Trunk vers HV (tous VLAN locaux)</t>
+          <t>Trunk vers HV (VLAN locaux + cluster/migration) — natif 997</t>
         </is>
       </c>
     </row>
@@ -21456,27 +21506,27 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>MGMT (VRF-MGMT)</t>
+          <t>MGMT (non raccordé)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>/24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>999</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -21486,7 +21536,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Accès admin</t>
+          <t>Interface OOB non câblée dans la maquette : administration via Loopback0</t>
         </is>
       </c>
     </row>
@@ -22158,7 +22208,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW ADMIN-MONITOR-PERF</t>
+          <t>Anycast GW ADMIN-OBSERV</t>
         </is>
       </c>
     </row>
@@ -22291,7 +22341,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Vlan400</t>
+          <t>Vlan306</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -22301,7 +22351,7 @@
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>10.5.0.1</t>
+          <t>10.4.36.1</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -22310,11 +22360,11 @@
         </is>
       </c>
       <c r="E41" s="10" t="n">
-        <v>400</v>
+        <v>306</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -22324,7 +22374,47 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW SOC-CORE</t>
+          <t>Anycast GW ADMIN-SOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Vlan999</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>SVI anycast gateway</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>10.254.0.1</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>/24</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>999</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Anycast GW MGMT-DC — passerelle des hyperviseurs</t>
         </is>
       </c>
     </row>
@@ -22339,7 +22429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22359,7 +22449,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -22475,8 +22564,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -22564,7 +22651,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Router-ID OSPF + source iBGP EVPN + VTEP</t>
+          <t>Router-ID OSPF + source iBGP EVPN + VTEP + administration in-band</t>
         </is>
       </c>
     </row>
@@ -22675,7 +22762,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>100-107,200-204,300-305,400,999</t>
+          <t>100-107,200-204,300-306,990,991,999</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -22690,7 +22777,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Trunk vers HV (tous VLAN locaux)</t>
+          <t>Trunk vers HV (VLAN locaux + cluster/migration) — natif 997</t>
         </is>
       </c>
     </row>
@@ -22702,27 +22789,27 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>MGMT (VRF-MGMT)</t>
+          <t>MGMT (non raccordé)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>10.254.0.12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>/24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>999</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>MGMT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -22732,7 +22819,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Accès admin</t>
+          <t>Interface OOB non câblée dans la maquette : administration via Loopback0</t>
         </is>
       </c>
     </row>
@@ -23404,7 +23491,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW ADMIN-MONITOR-PERF</t>
+          <t>Anycast GW ADMIN-OBSERV</t>
         </is>
       </c>
     </row>
@@ -23537,7 +23624,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Vlan400</t>
+          <t>Vlan306</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -23547,7 +23634,7 @@
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>10.5.0.1</t>
+          <t>10.4.36.1</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -23556,11 +23643,11 @@
         </is>
       </c>
       <c r="E41" s="10" t="n">
-        <v>400</v>
+        <v>306</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -23570,7 +23657,47 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Anycast GW SOC-CORE</t>
+          <t>Anycast GW ADMIN-SOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Vlan999</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>SVI anycast gateway</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>10.254.0.1</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>/24</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>999</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Anycast GW MGMT-DC — passerelle des hyperviseurs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-07-30 10:17:17
</commit_message>
<xml_diff>
--- a/cartographie.xlsx
+++ b/cartographie.xlsx
@@ -151,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,6 +200,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1669,7 +1672,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1761,8 +1763,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -2273,7 +2273,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2365,8 +2364,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -2877,7 +2874,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2969,8 +2965,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -3763,7 +3757,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3855,8 +3848,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -4649,7 +4640,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -4741,8 +4731,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -5535,7 +5523,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -5627,8 +5614,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -6421,7 +6406,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6513,8 +6497,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -6801,7 +6783,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6893,8 +6874,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -7181,7 +7160,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -7273,8 +7251,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -11442,7 +11418,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -11534,8 +11509,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -13418,7 +13391,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -13426,7 +13398,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -13637,8 +13608,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -14167,7 +14136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14179,6 +14148,9 @@
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14241,6 +14213,21 @@
           <t>Rôle</t>
         </is>
       </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>VNI L2</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>VNI L3</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>RD / RT</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -14286,6 +14273,21 @@
           <t>NAT Cloud libvirt ; subnet fusionné WAN + bloc public (VIP CARP services)</t>
         </is>
       </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -14331,6 +14333,21 @@
           <t>pfsync dédié FW-1 ↔ FW-2</t>
         </is>
       </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -14376,6 +14393,21 @@
           <t>Loopbacks équipements (/32 chacune)</t>
         </is>
       </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -14421,6 +14453,21 @@
           <t>SPINE-1 ↔ LEAF-1</t>
         </is>
       </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -14466,6 +14513,21 @@
           <t>SPINE-1 ↔ LEAF-2</t>
         </is>
       </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -14511,6 +14573,21 @@
           <t>SPINE-1 ↔ LEAF-3</t>
         </is>
       </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -14556,6 +14633,21 @@
           <t>SPINE-2 ↔ LEAF-1</t>
         </is>
       </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -14601,6 +14693,21 @@
           <t>SPINE-2 ↔ LEAF-2</t>
         </is>
       </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -14646,6 +14753,21 @@
           <t>SPINE-2 ↔ LEAF-3</t>
         </is>
       </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -14691,6 +14813,21 @@
           <t>FW-1 ↔ SPINE-1 (underlay)</t>
         </is>
       </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -14736,6 +14873,21 @@
           <t>FW-1 ↔ SPINE-2 (underlay)</t>
         </is>
       </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -14781,6 +14933,21 @@
           <t>FW-2 ↔ SPINE-1 (underlay)</t>
         </is>
       </c>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -14826,6 +14993,21 @@
           <t>FW-2 ↔ SPINE-2 (underlay)</t>
         </is>
       </c>
+      <c r="J17" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -14869,6 +15051,19 @@
           <t>Transit VRF-PROD FW ↔ Spine (VLAN 4001)</t>
         </is>
       </c>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L18" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -14912,6 +15107,19 @@
           <t>Transit VRF-DMZ FW ↔ Spine (VLAN 4002)</t>
         </is>
       </c>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L19" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -14955,6 +15163,19 @@
           <t>Transit VRF-ADMIN FW ↔ Spine (VLAN 4003)</t>
         </is>
       </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L20" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -14998,6 +15219,19 @@
           <t>Transit VRF-MGMT FW ↔ Spine (VLAN 4004)</t>
         </is>
       </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="19" t="n">
+        <v>50004</v>
+      </c>
+      <c r="L21" s="19" t="inlineStr">
+        <is>
+          <t>65000:999</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -15043,6 +15277,21 @@
           <t>FW-1 ↔ CORE-1</t>
         </is>
       </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -15088,6 +15337,21 @@
           <t>FW-1 ↔ CORE-2</t>
         </is>
       </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -15133,6 +15397,21 @@
           <t>FW-2 ↔ CORE-1</t>
         </is>
       </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -15178,6 +15457,21 @@
           <t>FW-2 ↔ CORE-2</t>
         </is>
       </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -15223,6 +15517,21 @@
           <t>CORE-1 ↔ DIST-1</t>
         </is>
       </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -15268,6 +15577,21 @@
           <t>CORE-1 ↔ DIST-2</t>
         </is>
       </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -15313,6 +15637,21 @@
           <t>CORE-1 ↔ DIST-3</t>
         </is>
       </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -15358,6 +15697,21 @@
           <t>CORE-1 ↔ DIST-4</t>
         </is>
       </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -15403,6 +15757,21 @@
           <t>CORE-2 ↔ DIST-1</t>
         </is>
       </c>
+      <c r="J30" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -15448,6 +15817,21 @@
           <t>CORE-2 ↔ DIST-2</t>
         </is>
       </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -15493,6 +15877,21 @@
           <t>CORE-2 ↔ DIST-3</t>
         </is>
       </c>
+      <c r="J32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -15538,6 +15937,21 @@
           <t>CORE-2 ↔ DIST-4</t>
         </is>
       </c>
+      <c r="J33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -15583,6 +15997,21 @@
           <t>USERS bloc 1</t>
         </is>
       </c>
+      <c r="J34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -15628,6 +16057,21 @@
           <t>VOICE bloc 1</t>
         </is>
       </c>
+      <c r="J35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -15673,6 +16117,21 @@
           <t>IOT bloc 1</t>
         </is>
       </c>
+      <c r="J36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -15718,6 +16177,21 @@
           <t>WIFI-CORP bloc 1</t>
         </is>
       </c>
+      <c r="J37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -15763,6 +16237,21 @@
           <t>WIFI-GUEST bloc 1</t>
         </is>
       </c>
+      <c r="J38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -15808,6 +16297,21 @@
           <t>WIFI-BYOD bloc 1</t>
         </is>
       </c>
+      <c r="J39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -15853,6 +16357,21 @@
           <t>PRINTERS bloc 1</t>
         </is>
       </c>
+      <c r="J40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -15898,6 +16417,21 @@
           <t>LAB-DEV bloc 1</t>
         </is>
       </c>
+      <c r="J41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -15943,6 +16477,21 @@
           <t>USERS bloc 2</t>
         </is>
       </c>
+      <c r="J42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -15988,6 +16537,21 @@
           <t>VOICE bloc 2</t>
         </is>
       </c>
+      <c r="J43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -16033,6 +16597,21 @@
           <t>IOT bloc 2</t>
         </is>
       </c>
+      <c r="J44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -16078,6 +16657,21 @@
           <t>WIFI-CORP bloc 2</t>
         </is>
       </c>
+      <c r="J45" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -16123,6 +16717,21 @@
           <t>WIFI-GUEST bloc 2</t>
         </is>
       </c>
+      <c r="J46" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -16168,6 +16777,21 @@
           <t>WIFI-BYOD bloc 2</t>
         </is>
       </c>
+      <c r="J47" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
@@ -16213,6 +16837,21 @@
           <t>PRINTERS bloc 2</t>
         </is>
       </c>
+      <c r="J48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
@@ -16258,6 +16897,21 @@
           <t>LAB-DEV bloc 2</t>
         </is>
       </c>
+      <c r="J49" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
@@ -16303,6 +16957,17 @@
           <t>PROD-WEB-INT (Anycast GW)</t>
         </is>
       </c>
+      <c r="J50" s="19" t="n">
+        <v>10100</v>
+      </c>
+      <c r="K50" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L50" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
@@ -16348,6 +17013,17 @@
           <t>PROD-APP</t>
         </is>
       </c>
+      <c r="J51" s="19" t="n">
+        <v>10101</v>
+      </c>
+      <c r="K51" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L51" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
@@ -16393,6 +17069,17 @@
           <t>PROD-DB</t>
         </is>
       </c>
+      <c r="J52" s="19" t="n">
+        <v>10102</v>
+      </c>
+      <c r="K52" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L52" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n">
@@ -16438,6 +17125,17 @@
           <t>PROD-INFRA</t>
         </is>
       </c>
+      <c r="J53" s="19" t="n">
+        <v>10103</v>
+      </c>
+      <c r="K53" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L53" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
@@ -16483,6 +17181,17 @@
           <t>PROD-FILES</t>
         </is>
       </c>
+      <c r="J54" s="19" t="n">
+        <v>10104</v>
+      </c>
+      <c r="K54" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L54" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n">
@@ -16528,6 +17237,17 @@
           <t>PROD-MESSAGING</t>
         </is>
       </c>
+      <c r="J55" s="19" t="n">
+        <v>10105</v>
+      </c>
+      <c r="K55" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L55" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
@@ -16573,6 +17293,17 @@
           <t>PROD-TOIP</t>
         </is>
       </c>
+      <c r="J56" s="19" t="n">
+        <v>10106</v>
+      </c>
+      <c r="K56" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L56" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n">
@@ -16618,6 +17349,17 @@
           <t>PROD-INTEGRATION</t>
         </is>
       </c>
+      <c r="J57" s="19" t="n">
+        <v>10107</v>
+      </c>
+      <c r="K57" s="19" t="n">
+        <v>50001</v>
+      </c>
+      <c r="L57" s="19" t="inlineStr">
+        <is>
+          <t>65000:100</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
@@ -16663,6 +17405,17 @@
           <t>DMZ-FRONT</t>
         </is>
       </c>
+      <c r="J58" s="19" t="n">
+        <v>10200</v>
+      </c>
+      <c r="K58" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L58" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
@@ -16708,6 +17461,17 @@
           <t>DMZ-WEB</t>
         </is>
       </c>
+      <c r="J59" s="19" t="n">
+        <v>10201</v>
+      </c>
+      <c r="K59" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L59" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
@@ -16753,6 +17517,17 @@
           <t>DMZ-MAIL</t>
         </is>
       </c>
+      <c r="J60" s="19" t="n">
+        <v>10202</v>
+      </c>
+      <c r="K60" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L60" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n">
@@ -16798,6 +17573,17 @@
           <t>DMZ-DNS</t>
         </is>
       </c>
+      <c r="J61" s="19" t="n">
+        <v>10203</v>
+      </c>
+      <c r="K61" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L61" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -16843,6 +17629,17 @@
           <t>DMZ-API</t>
         </is>
       </c>
+      <c r="J62" s="19" t="n">
+        <v>10204</v>
+      </c>
+      <c r="K62" s="19" t="n">
+        <v>50002</v>
+      </c>
+      <c r="L62" s="19" t="inlineStr">
+        <is>
+          <t>65000:200</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n">
@@ -16888,6 +17685,17 @@
           <t>ADMIN-CORE (bastion, PBS, PDM)</t>
         </is>
       </c>
+      <c r="J63" s="19" t="n">
+        <v>10300</v>
+      </c>
+      <c r="K63" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L63" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
@@ -16933,6 +17741,17 @@
           <t>ADMIN-CICD (GitLab, Jenkins)</t>
         </is>
       </c>
+      <c r="J64" s="19" t="n">
+        <v>10301</v>
+      </c>
+      <c r="K64" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L64" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
@@ -16978,6 +17797,17 @@
           <t>ADMIN-OBSERV (Alloy, Prometheus, Loki, Tempo, Grafana)</t>
         </is>
       </c>
+      <c r="J65" s="19" t="n">
+        <v>10302</v>
+      </c>
+      <c r="K65" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L65" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -17023,6 +17853,17 @@
           <t>ADMIN-AAA (FreeRADIUS, Keycloak)</t>
         </is>
       </c>
+      <c r="J66" s="19" t="n">
+        <v>10303</v>
+      </c>
+      <c r="K66" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L66" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
@@ -17068,6 +17909,17 @@
           <t>ADMIN-AUTOMATE (Ansible)</t>
         </is>
       </c>
+      <c r="J67" s="19" t="n">
+        <v>10304</v>
+      </c>
+      <c r="K67" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L67" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
@@ -17113,6 +17965,17 @@
           <t>ADMIN-VAULT</t>
         </is>
       </c>
+      <c r="J68" s="19" t="n">
+        <v>10305</v>
+      </c>
+      <c r="K68" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L68" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
@@ -17156,6 +18019,17 @@
           <t>ADMIN-SOC (Wazuh, MISP, DFIR-IRIS, Shuffle, Malcolm)</t>
         </is>
       </c>
+      <c r="J69" s="19" t="n">
+        <v>10306</v>
+      </c>
+      <c r="K69" s="19" t="n">
+        <v>50003</v>
+      </c>
+      <c r="L69" s="19" t="inlineStr">
+        <is>
+          <t>65000:300</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
@@ -17199,6 +18073,17 @@
           <t>MGMT-DC — interfaces d'administration des hyperviseurs (VNI 10999)</t>
         </is>
       </c>
+      <c r="J70" s="19" t="n">
+        <v>10999</v>
+      </c>
+      <c r="K70" s="19" t="n">
+        <v>50004</v>
+      </c>
+      <c r="L70" s="19" t="inlineStr">
+        <is>
+          <t>65000:999</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
@@ -17242,6 +18127,21 @@
           <t>MGMT-LAN bloc 1 — SVI des ACC-1/ACC-2, passerelle sur DIST-1/DIST-2</t>
         </is>
       </c>
+      <c r="J71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -17285,6 +18185,21 @@
           <t>MGMT-LAN bloc 2 — SVI des ACC-3/ACC-4, passerelle sur DIST-3/DIST-4</t>
         </is>
       </c>
+      <c r="J72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17294,6 +18209,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A74:L74"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>